<commit_message>
Expand Ask Ekiti tourism culture and health coverage
</commit_message>
<xml_diff>
--- a/14_Source_Documents/Ask_Ekiti_Source_Inventory.xlsx
+++ b/14_Source_Documents/Ask_Ekiti_Source_Inventory.xlsx
@@ -847,7 +847,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:Y319"/>
+  <dimension ref="A1:Y323"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="28" min="1" max="1"/>
@@ -6013,6 +6013,362 @@
       <c r="V319" s="28" t="inlineStr">
         <is>
           <t>02_LGAs/lga-*.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" s="28" t="inlineStr">
+        <is>
+          <t>SRC-047</t>
+        </is>
+      </c>
+      <c r="B320" s="28" t="inlineStr">
+        <is>
+          <t>Identified</t>
+        </is>
+      </c>
+      <c r="C320" s="28" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D320" s="28" t="inlineStr">
+        <is>
+          <t>tourism</t>
+        </is>
+      </c>
+      <c r="E320" s="28" t="inlineStr">
+        <is>
+          <t>Arinta Waterfall location, Ramsar designation and ecological characteristics</t>
+        </is>
+      </c>
+      <c r="F320" s="28" t="inlineStr">
+        <is>
+          <t>RIS for Site no. 2565, Arinta Waterfall, Nigeria</t>
+        </is>
+      </c>
+      <c r="G320" s="28" t="inlineStr">
+        <is>
+          <t>International treaty registry / official wetland information sheet</t>
+        </is>
+      </c>
+      <c r="H320" s="28" t="inlineStr">
+        <is>
+          <t>Primary (official)</t>
+        </is>
+      </c>
+      <c r="I320" s="28" t="inlineStr">
+        <is>
+          <t>Ramsar Sites Information Service</t>
+        </is>
+      </c>
+      <c r="J320" s="28" t="inlineStr">
+        <is>
+          <t>https://rsis.ramsar.org/RISapp/files/RISrep/NG2565RIS_2503_en.pdf</t>
+        </is>
+      </c>
+      <c r="K320" s="28" t="inlineStr">
+        <is>
+          <t>Official international registry</t>
+        </is>
+      </c>
+      <c r="M320" s="28" t="n"/>
+      <c r="N320" s="28" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O320" s="28" t="inlineStr">
+        <is>
+          <t>Culture &amp; Tourism</t>
+        </is>
+      </c>
+      <c r="P320" s="28" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="T320" t="inlineStr">
+        <is>
+          <t>Official Ramsar Site 2565 record for Arinta Waterfall.</t>
+        </is>
+      </c>
+      <c r="U320" s="28" t="n"/>
+      <c r="V320" s="28" t="inlineStr">
+        <is>
+          <t>04_Tourism/arinta-waterfall.md</t>
+        </is>
+      </c>
+      <c r="W320" t="inlineStr">
+        <is>
+          <t>04_Tourism/arinta-waterfall.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" s="28" t="inlineStr">
+        <is>
+          <t>SRC-048</t>
+        </is>
+      </c>
+      <c r="B321" s="28" t="inlineStr">
+        <is>
+          <t>Identified</t>
+        </is>
+      </c>
+      <c r="C321" s="28" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D321" s="28" t="inlineStr">
+        <is>
+          <t>culture</t>
+        </is>
+      </c>
+      <c r="E321" s="28" t="inlineStr">
+        <is>
+          <t>Udiroko Festival existence, activities and cultural role</t>
+        </is>
+      </c>
+      <c r="F321" s="28" t="inlineStr">
+        <is>
+          <t>Udiroko Festival: A Catalyst For Development</t>
+        </is>
+      </c>
+      <c r="G321" s="28" t="inlineStr">
+        <is>
+          <t>Government article</t>
+        </is>
+      </c>
+      <c r="H321" s="28" t="inlineStr">
+        <is>
+          <t>Primary (official)</t>
+        </is>
+      </c>
+      <c r="I321" s="28" t="inlineStr">
+        <is>
+          <t>Government of Ekiti State</t>
+        </is>
+      </c>
+      <c r="J321" s="28" t="inlineStr">
+        <is>
+          <t>https://www.ekitistate.gov.ng/archives/4314</t>
+        </is>
+      </c>
+      <c r="K321" s="28" t="inlineStr">
+        <is>
+          <t>Official government website</t>
+        </is>
+      </c>
+      <c r="M321" s="28" t="n"/>
+      <c r="N321" s="28" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O321" s="28" t="inlineStr">
+        <is>
+          <t>Culture &amp; Tourism</t>
+        </is>
+      </c>
+      <c r="P321" s="28" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="T321" t="inlineStr">
+        <is>
+          <t>Official Ekiti State Government article on Udiroko Festival.</t>
+        </is>
+      </c>
+      <c r="U321" s="28" t="n"/>
+      <c r="V321" s="28" t="inlineStr">
+        <is>
+          <t>05_Culture/udiroko-festival.md</t>
+        </is>
+      </c>
+      <c r="W321" t="inlineStr">
+        <is>
+          <t>05_Culture/udiroko-festival.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" s="28" t="inlineStr">
+        <is>
+          <t>SRC-049</t>
+        </is>
+      </c>
+      <c r="B322" s="28" t="inlineStr">
+        <is>
+          <t>Identified</t>
+        </is>
+      </c>
+      <c r="C322" s="28" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D322" s="28" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="E322" s="28" t="inlineStr">
+        <is>
+          <t>Ekiti State Health Insurance Scheme and Ulerawa health-insurance context</t>
+        </is>
+      </c>
+      <c r="F322" s="28" t="inlineStr">
+        <is>
+          <t>Ekiti State Health Insurance Scheme</t>
+        </is>
+      </c>
+      <c r="G322" s="28" t="inlineStr">
+        <is>
+          <t>Government MDA webpage</t>
+        </is>
+      </c>
+      <c r="H322" s="28" t="inlineStr">
+        <is>
+          <t>Primary (official)</t>
+        </is>
+      </c>
+      <c r="I322" s="28" t="inlineStr">
+        <is>
+          <t>Government of Ekiti State</t>
+        </is>
+      </c>
+      <c r="J322" s="28" t="inlineStr">
+        <is>
+          <t>https://www.ekitistate.gov.ng/executive-council/mdas/ekiti-state-health-insurance-scheme</t>
+        </is>
+      </c>
+      <c r="K322" s="28" t="inlineStr">
+        <is>
+          <t>Official government website</t>
+        </is>
+      </c>
+      <c r="M322" s="28" t="n"/>
+      <c r="N322" s="28" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O322" s="28" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="P322" s="28" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="T322" t="inlineStr">
+        <is>
+          <t>Official Ekiti State Government health-insurance page.</t>
+        </is>
+      </c>
+      <c r="U322" s="28" t="n"/>
+      <c r="V322" s="28" t="inlineStr">
+        <is>
+          <t>07_Health/programmes/EK-HEA-PROG-001_Ulerawa_Health_Programme.md</t>
+        </is>
+      </c>
+      <c r="W322" t="inlineStr">
+        <is>
+          <t>07_Health/programmes/EK-HEA-PROG-001_Ulerawa_Health_Programme.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" s="28" t="inlineStr">
+        <is>
+          <t>SRC-050</t>
+        </is>
+      </c>
+      <c r="B323" s="28" t="inlineStr">
+        <is>
+          <t>Identified</t>
+        </is>
+      </c>
+      <c r="C323" s="28" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D323" s="28" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="E323" s="28" t="inlineStr">
+        <is>
+          <t>Ulerawa programme services, reach and reported beneficiary figures</t>
+        </is>
+      </c>
+      <c r="F323" s="28" t="inlineStr">
+        <is>
+          <t>Over 429,000 Residents Benefit From Ekiti Govt’s Free Health Programme</t>
+        </is>
+      </c>
+      <c r="G323" s="28" t="inlineStr">
+        <is>
+          <t>Government programme update</t>
+        </is>
+      </c>
+      <c r="H323" s="28" t="inlineStr">
+        <is>
+          <t>Primary (official)</t>
+        </is>
+      </c>
+      <c r="I323" s="28" t="inlineStr">
+        <is>
+          <t>Government of Ekiti State</t>
+        </is>
+      </c>
+      <c r="J323" s="28" t="inlineStr">
+        <is>
+          <t>https://www.ekitistate.gov.ng/archives/29019</t>
+        </is>
+      </c>
+      <c r="K323" s="28" t="inlineStr">
+        <is>
+          <t>Official government website</t>
+        </is>
+      </c>
+      <c r="M323" s="28" t="n"/>
+      <c r="N323" s="28" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O323" s="28" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="P323" s="28" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="T323" t="inlineStr">
+        <is>
+          <t>Official state programme update. Numerical claims must retain their date and attribution.</t>
+        </is>
+      </c>
+      <c r="U323" s="28" t="n"/>
+      <c r="V323" s="28" t="inlineStr">
+        <is>
+          <t>07_Health/programmes/EK-HEA-PROG-001_Ulerawa_Health_Programme.md</t>
+        </is>
+      </c>
+      <c r="W323" t="inlineStr">
+        <is>
+          <t>07_Health/programmes/EK-HEA-PROG-001_Ulerawa_Health_Programme.md</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Normalize first Ask Ekiti education sources
</commit_message>
<xml_diff>
--- a/14_Source_Documents/Ask_Ekiti_Source_Inventory.xlsx
+++ b/14_Source_Documents/Ask_Ekiti_Source_Inventory.xlsx
@@ -847,7 +847,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:Y323"/>
+  <dimension ref="A1:Y326"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="28" min="1" max="1"/>
@@ -6088,7 +6088,7 @@
           <t>Needs review</t>
         </is>
       </c>
-      <c r="T320" t="inlineStr">
+      <c r="T320" s="0" t="inlineStr">
         <is>
           <t>Official Ramsar Site 2565 record for Arinta Waterfall.</t>
         </is>
@@ -6099,7 +6099,7 @@
           <t>04_Tourism/arinta-waterfall.md</t>
         </is>
       </c>
-      <c r="W320" t="inlineStr">
+      <c r="W320" s="0" t="inlineStr">
         <is>
           <t>04_Tourism/arinta-waterfall.md</t>
         </is>
@@ -6177,7 +6177,7 @@
           <t>Needs review</t>
         </is>
       </c>
-      <c r="T321" t="inlineStr">
+      <c r="T321" s="0" t="inlineStr">
         <is>
           <t>Official Ekiti State Government article on Udiroko Festival.</t>
         </is>
@@ -6188,7 +6188,7 @@
           <t>05_Culture/udiroko-festival.md</t>
         </is>
       </c>
-      <c r="W321" t="inlineStr">
+      <c r="W321" s="0" t="inlineStr">
         <is>
           <t>05_Culture/udiroko-festival.md</t>
         </is>
@@ -6266,7 +6266,7 @@
           <t>Needs review</t>
         </is>
       </c>
-      <c r="T322" t="inlineStr">
+      <c r="T322" s="0" t="inlineStr">
         <is>
           <t>Official Ekiti State Government health-insurance page.</t>
         </is>
@@ -6277,7 +6277,7 @@
           <t>07_Health/programmes/EK-HEA-PROG-001_Ulerawa_Health_Programme.md</t>
         </is>
       </c>
-      <c r="W322" t="inlineStr">
+      <c r="W322" s="0" t="inlineStr">
         <is>
           <t>07_Health/programmes/EK-HEA-PROG-001_Ulerawa_Health_Programme.md</t>
         </is>
@@ -6355,7 +6355,7 @@
           <t>Needs review</t>
         </is>
       </c>
-      <c r="T323" t="inlineStr">
+      <c r="T323" s="0" t="inlineStr">
         <is>
           <t>Official state programme update. Numerical claims must retain their date and attribution.</t>
         </is>
@@ -6366,9 +6366,280 @@
           <t>07_Health/programmes/EK-HEA-PROG-001_Ulerawa_Health_Programme.md</t>
         </is>
       </c>
-      <c r="W323" t="inlineStr">
+      <c r="W323" s="0" t="inlineStr">
         <is>
           <t>07_Health/programmes/EK-HEA-PROG-001_Ulerawa_Health_Programme.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" s="28" t="inlineStr">
+        <is>
+          <t>SRC-051</t>
+        </is>
+      </c>
+      <c r="B324" s="28" t="inlineStr">
+        <is>
+          <t>Identified</t>
+        </is>
+      </c>
+      <c r="C324" s="28" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D324" s="28" t="inlineStr">
+        <is>
+          <t>education</t>
+        </is>
+      </c>
+      <c r="E324" s="28" t="inlineStr">
+        <is>
+          <t>Afe Babalola University founder, 1 October 2008 turning of the sod, and May 2009 NUC assessment visit</t>
+        </is>
+      </c>
+      <c r="F324" s="28" t="inlineStr">
+        <is>
+          <t>Office of the Founder</t>
+        </is>
+      </c>
+      <c r="G324" s="28" t="inlineStr">
+        <is>
+          <t>University official webpage</t>
+        </is>
+      </c>
+      <c r="H324" s="28" t="inlineStr">
+        <is>
+          <t>Primary (official)</t>
+        </is>
+      </c>
+      <c r="I324" s="28" t="inlineStr">
+        <is>
+          <t>Afe Babalola University</t>
+        </is>
+      </c>
+      <c r="J324" s="28" t="inlineStr">
+        <is>
+          <t>https://www.abuad.edu.ng/office-of-the-founder/</t>
+        </is>
+      </c>
+      <c r="K324" s="28" t="inlineStr">
+        <is>
+          <t>Official university website</t>
+        </is>
+      </c>
+      <c r="M324" s="28" t="n"/>
+      <c r="N324" s="28" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O324" s="28" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="P324" s="28" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="T324" s="0" t="inlineStr">
+        <is>
+          <t>Official ABUAD institutional source used for the university's founding history.</t>
+        </is>
+      </c>
+      <c r="U324" s="28" t="n"/>
+      <c r="V324" s="28" t="inlineStr">
+        <is>
+          <t>06_Education/institutions/abuad/metadata.md</t>
+        </is>
+      </c>
+      <c r="W324" s="0" t="inlineStr">
+        <is>
+          <t>06_Education/institutions/abuad/metadata.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" s="28" t="inlineStr">
+        <is>
+          <t>SRC-052</t>
+        </is>
+      </c>
+      <c r="B325" s="28" t="inlineStr">
+        <is>
+          <t>Identified</t>
+        </is>
+      </c>
+      <c r="C325" s="28" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D325" s="28" t="inlineStr">
+        <is>
+          <t>education</t>
+        </is>
+      </c>
+      <c r="E325" s="28" t="inlineStr">
+        <is>
+          <t>Ekiti State University establishment and institutional name history</t>
+        </is>
+      </c>
+      <c r="F325" s="28" t="inlineStr">
+        <is>
+          <t>About EKSU</t>
+        </is>
+      </c>
+      <c r="G325" s="28" t="inlineStr">
+        <is>
+          <t>University official webpage</t>
+        </is>
+      </c>
+      <c r="H325" s="28" t="inlineStr">
+        <is>
+          <t>Primary (official)</t>
+        </is>
+      </c>
+      <c r="I325" s="28" t="inlineStr">
+        <is>
+          <t>Ekiti State University</t>
+        </is>
+      </c>
+      <c r="J325" s="28" t="inlineStr">
+        <is>
+          <t>https://eksu.edu.ng/about-eksu/</t>
+        </is>
+      </c>
+      <c r="K325" s="28" t="inlineStr">
+        <is>
+          <t>Official university website</t>
+        </is>
+      </c>
+      <c r="M325" s="28" t="n"/>
+      <c r="N325" s="28" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O325" s="28" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="P325" s="28" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="T325" s="0" t="inlineStr">
+        <is>
+          <t>Official EKSU institutional history page.</t>
+        </is>
+      </c>
+      <c r="U325" s="28" t="n"/>
+      <c r="V325" s="28" t="inlineStr">
+        <is>
+          <t>06_Education/institutions/eksu/metadata.md</t>
+        </is>
+      </c>
+      <c r="W325" s="0" t="inlineStr">
+        <is>
+          <t>06_Education/institutions/eksu/metadata.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" s="28" t="inlineStr">
+        <is>
+          <t>SRC-053</t>
+        </is>
+      </c>
+      <c r="B326" s="28" t="inlineStr">
+        <is>
+          <t>Identified</t>
+        </is>
+      </c>
+      <c r="C326" s="28" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D326" s="28" t="inlineStr">
+        <is>
+          <t>education</t>
+        </is>
+      </c>
+      <c r="E326" s="28" t="inlineStr">
+        <is>
+          <t>Federal Polytechnic Ado-Ekiti official federal-polytechnic status and establishment year 1977</t>
+        </is>
+      </c>
+      <c r="F326" s="28" t="inlineStr">
+        <is>
+          <t>Federal Polytechnics</t>
+        </is>
+      </c>
+      <c r="G326" s="28" t="inlineStr">
+        <is>
+          <t>Federal government education directory</t>
+        </is>
+      </c>
+      <c r="H326" s="28" t="inlineStr">
+        <is>
+          <t>Primary (official)</t>
+        </is>
+      </c>
+      <c r="I326" s="28" t="inlineStr">
+        <is>
+          <t>Federal Ministry of Education</t>
+        </is>
+      </c>
+      <c r="J326" s="28" t="inlineStr">
+        <is>
+          <t>https://education.gov.ng/government-polytechnics/</t>
+        </is>
+      </c>
+      <c r="K326" s="28" t="inlineStr">
+        <is>
+          <t>Official federal government website</t>
+        </is>
+      </c>
+      <c r="M326" s="28" t="n"/>
+      <c r="N326" s="28" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O326" s="28" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="P326" s="28" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="T326" s="0" t="inlineStr">
+        <is>
+          <t>Official Federal Ministry of Education directory entry.</t>
+        </is>
+      </c>
+      <c r="U326" s="28" t="inlineStr">
+        <is>
+          <t>This source is used only for institution status and establishment year; relocation-history claims require a separate source.</t>
+        </is>
+      </c>
+      <c r="V326" s="28" t="inlineStr">
+        <is>
+          <t>06_Education/institutions/fedpoly-ado-ekiti/metadata.md</t>
+        </is>
+      </c>
+      <c r="W326" s="0" t="inlineStr">
+        <is>
+          <t>06_Education/institutions/fedpoly-ado-ekiti/metadata.md</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Normalize FUTES Ask Ekiti education record
</commit_message>
<xml_diff>
--- a/14_Source_Documents/Ask_Ekiti_Source_Inventory.xlsx
+++ b/14_Source_Documents/Ask_Ekiti_Source_Inventory.xlsx
@@ -847,7 +847,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:Y326"/>
+  <dimension ref="A1:Y327"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="28" min="1" max="1"/>
@@ -6640,6 +6640,99 @@
       <c r="W326" s="0" t="inlineStr">
         <is>
           <t>06_Education/institutions/fedpoly-ado-ekiti/metadata.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" s="28" t="inlineStr">
+        <is>
+          <t>SRC-054</t>
+        </is>
+      </c>
+      <c r="B327" s="28" t="inlineStr">
+        <is>
+          <t>Identified</t>
+        </is>
+      </c>
+      <c r="C327" s="28" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D327" s="28" t="inlineStr">
+        <is>
+          <t>education</t>
+        </is>
+      </c>
+      <c r="E327" s="28" t="inlineStr">
+        <is>
+          <t>FUTES establishment date, legislative history and pioneer management</t>
+        </is>
+      </c>
+      <c r="F327" s="28" t="inlineStr">
+        <is>
+          <t>History</t>
+        </is>
+      </c>
+      <c r="G327" s="28" t="inlineStr">
+        <is>
+          <t>University official webpage</t>
+        </is>
+      </c>
+      <c r="H327" s="28" t="inlineStr">
+        <is>
+          <t>Primary (official)</t>
+        </is>
+      </c>
+      <c r="I327" s="28" t="inlineStr">
+        <is>
+          <t>Federal University of Technology and Environmental Sciences (FUTES), Iyin-Ekiti</t>
+        </is>
+      </c>
+      <c r="J327" s="28" t="inlineStr">
+        <is>
+          <t>https://futes.edu.ng/history</t>
+        </is>
+      </c>
+      <c r="K327" s="28" t="inlineStr">
+        <is>
+          <t>Official university website</t>
+        </is>
+      </c>
+      <c r="M327" s="28" t="n"/>
+      <c r="N327" s="28" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O327" s="28" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="P327" s="28" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="T327" s="0" t="inlineStr">
+        <is>
+          <t>Official FUTES institutional history page used for establishment and pioneer-management facts.</t>
+        </is>
+      </c>
+      <c r="U327" s="28" t="inlineStr">
+        <is>
+          <t>Fast-changing claims such as admissions and accreditation are excluded.</t>
+        </is>
+      </c>
+      <c r="V327" s="28" t="inlineStr">
+        <is>
+          <t>06_Education/institutions/futes-iyin-ekiti/metadata.md</t>
+        </is>
+      </c>
+      <c r="W327" s="0" t="inlineStr">
+        <is>
+          <t>06_Education/institutions/futes-iyin-ekiti/metadata.md</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Normalize EKSPOLY Ask Ekiti education record
</commit_message>
<xml_diff>
--- a/14_Source_Documents/Ask_Ekiti_Source_Inventory.xlsx
+++ b/14_Source_Documents/Ask_Ekiti_Source_Inventory.xlsx
@@ -847,7 +847,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:Y327"/>
+  <dimension ref="A1:Y328"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="28" min="1" max="1"/>
@@ -6733,6 +6733,103 @@
       <c r="W327" s="0" t="inlineStr">
         <is>
           <t>06_Education/institutions/futes-iyin-ekiti/metadata.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" s="28" t="inlineStr">
+        <is>
+          <t>SRC-055</t>
+        </is>
+      </c>
+      <c r="B328" s="28" t="inlineStr">
+        <is>
+          <t>Identified</t>
+        </is>
+      </c>
+      <c r="C328" s="28" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D328" s="28" t="inlineStr">
+        <is>
+          <t>education</t>
+        </is>
+      </c>
+      <c r="E328" s="28" t="inlineStr">
+        <is>
+          <t>Ekiti State Polytechnic, Isan-Ekiti legal history; 2019 principal law and 2021 renaming to Ekiti State Polytechnic</t>
+        </is>
+      </c>
+      <c r="F328" s="28" t="inlineStr">
+        <is>
+          <t>Ekiti State Polytechnic, Isan-Ekiti (Second Amendment) Law, 2021</t>
+        </is>
+      </c>
+      <c r="G328" s="28" t="inlineStr">
+        <is>
+          <t>State law / official legislative document</t>
+        </is>
+      </c>
+      <c r="H328" s="28" t="inlineStr">
+        <is>
+          <t>Primary (official)</t>
+        </is>
+      </c>
+      <c r="I328" s="28" t="inlineStr">
+        <is>
+          <t>Ekiti State House of Assembly</t>
+        </is>
+      </c>
+      <c r="J328" s="28" t="inlineStr">
+        <is>
+          <t>https://hoa.ekitistate.gov.ng/dashboard/doc/No.%2018%20of%202021%20-%20EKITI%20STATE%20COLLEGE%20OF%20AGRICULTURE%20AND%20TECHNOLOGY.pdf</t>
+        </is>
+      </c>
+      <c r="K328" s="28" t="inlineStr">
+        <is>
+          <t>Official state legislature website</t>
+        </is>
+      </c>
+      <c r="M328" s="28" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="N328" s="28" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O328" s="28" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="P328" s="28" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="T328" s="0" t="inlineStr">
+        <is>
+          <t>Official state law identifying Law No. 6 of 2019 as the principal law and changing the institution's name to Ekiti State Polytechnic, Isan-Ekiti.</t>
+        </is>
+      </c>
+      <c r="U328" s="28" t="inlineStr">
+        <is>
+          <t>Do not use this source for the unsupported 2014 founding claim.</t>
+        </is>
+      </c>
+      <c r="V328" s="28" t="inlineStr">
+        <is>
+          <t>06_Education/institutions/ekspoly-isan-ekiti/metadata.md</t>
+        </is>
+      </c>
+      <c r="W328" s="0" t="inlineStr">
+        <is>
+          <t>06_Education/institutions/ekspoly-isan-ekiti/metadata.md</t>
         </is>
       </c>
     </row>

</xml_diff>